<commit_message>
fix(CASE_D1): final evidence-alignment cleanup — resolve participant count, stale candidate-theme counts, and fallback tokens
</commit_message>
<xml_diff>
--- a/analysis/CASE_D1/CASE_D1_participant_workbook.xlsx
+++ b/analysis/CASE_D1/CASE_D1_participant_workbook.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,17 +522,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>D1_M03</t>
+          <t>D1_M02</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>HWCH3AR.docx</t>
+          <t>HWCH2AR.docx</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -541,36 +541,28 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>20413</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>general_response;healthcare_worker_wellbeing;awareness_education;healthcare_system_critique;training_deficit</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>D1_M04</t>
+          <t>D1_M03</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HWCH4AR.docx</t>
+          <t>HWCH3AR.docx</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -579,36 +571,36 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>15191</v>
+        <v>20413</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>general_response;professional_identity</t>
+          <t>general_response;healthcare_worker_wellbeing;awareness_education;healthcare_system_critique;training_deficit</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>D1_M05</t>
+          <t>D1_M04</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>HWCH6AR.docx</t>
+          <t>HWCH4AR.docx</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -617,36 +609,36 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>4</v>
+        <v>43</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>766</v>
+        <v>15191</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>general_response</t>
+          <t>general_response;professional_identity</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>D1_M06</t>
+          <t>D1_M05</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>HWCH7AR.docx</t>
+          <t>HWCH6AR.docx</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -655,14 +647,14 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>6110</v>
+        <v>766</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -674,17 +666,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>D1_M07</t>
+          <t>D1_M06</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>HWCH10AR.docx</t>
+          <t>HWCH7AR.docx</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -693,26 +685,26 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>380</v>
+        <v>6110</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Q2;Q3</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>contentment_as_core;safety_security;spiritual_moral_anchor</t>
+          <t>general_response</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>D1_M08</t>
+          <t>D1_M07</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -734,61 +726,61 @@
         <v>2</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q2;Q3</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>healthcare_system_critique;hidden_masked_distress;practical_recommendation;professional_identity;service_recipient_voice</t>
+          <t>contentment_as_core;safety_security;spiritual_moral_anchor</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>D1_P01</t>
+          <t>D1_M08</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>HWCH0AR.docx</t>
+          <t>HWCH10AR.docx</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>participant</t>
+          <t>moderator</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>120</v>
+        <v>2</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>15833</v>
+        <v>384</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q5</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>general_response;practical_recommendation;school_clinical_link;spiritual_moral_anchor;family_support_ecology</t>
+          <t>healthcare_system_critique;hidden_masked_distress;practical_recommendation;professional_identity;service_recipient_voice</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>D1_P02</t>
+          <t>D1_P01</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -807,10 +799,10 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>192</v>
+        <v>120</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>19700</v>
+        <v>15833</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -819,14 +811,14 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>general_response;school_clinical_link;practical_recommendation;awareness_education;service_recipient_voice</t>
+          <t>general_response;practical_recommendation;school_clinical_link;spiritual_moral_anchor;family_support_ecology</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>D1_P03</t>
+          <t>D1_P02</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -845,10 +837,10 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>102</v>
+        <v>192</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>13163</v>
+        <v>19700</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -857,14 +849,14 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>general_response;spiritual_moral_anchor;awareness_education;healthcare_system_critique;pillar_physical</t>
+          <t>general_response;school_clinical_link;practical_recommendation;awareness_education;service_recipient_voice</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>D1_P04</t>
+          <t>D1_P03</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -883,26 +875,26 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>37</v>
+        <v>102</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>6280</v>
+        <v>13163</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q1;Q2;Q3;Q5</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>general_response;family_support_ecology;practical_recommendation;child_vulnerability;training_deficit</t>
+          <t>general_response;spiritual_moral_anchor;awareness_education;healthcare_system_critique;pillar_physical</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>D1_P05</t>
+          <t>D1_P04</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -921,36 +913,36 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>2032</v>
+        <v>6280</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>general_response;practical_recommendation;spiritual_moral_anchor;balance_multidimensional</t>
+          <t>general_response;family_support_ecology;practical_recommendation;child_vulnerability;training_deficit</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>D1_P06</t>
+          <t>D1_P05</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>HWCH2AR.docx</t>
+          <t>HWCH0AR.docx</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -962,23 +954,23 @@
         <v>25</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>10255</v>
+        <v>2032</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q1;Q2;Q3</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>general_response;healthcare_system_critique;family_support_ecology</t>
+          <t>general_response;practical_recommendation;spiritual_moral_anchor;balance_multidimensional</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>D1_P07</t>
+          <t>D1_P06</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -997,14 +989,14 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>18975</v>
+        <v>10255</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1016,17 +1008,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>D1_P08</t>
+          <t>D1_P07</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>HWCH4AR.docx</t>
+          <t>HWCH2AR.docx</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1035,26 +1027,26 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2</v>
+        <v>47</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>985</v>
+        <v>18975</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>general_response</t>
+          <t>general_response;healthcare_system_critique;family_support_ecology</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>D1_P09</t>
+          <t>D1_P08</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1073,14 +1065,14 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>923</v>
+        <v>985</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Q3;Q6;Q7</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1092,17 +1084,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>D1_P10</t>
+          <t>D1_P09</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>HWCH6AR.docx</t>
+          <t>HWCH4AR.docx</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1111,26 +1103,26 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>26630</v>
+        <v>923</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4;Q5;Q6</t>
+          <t>Q3;Q6;Q7</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>general_response;cultural_local_adaptation;healthcare_system_critique;pillar_emotional;interdependent_care</t>
+          <t>general_response</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>D1_P11</t>
+          <t>D1_P10</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1149,26 +1141,26 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>9126</v>
+        <v>26630</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Q3;Q5</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q6</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>general_response;balance_multidimensional</t>
+          <t>general_response;cultural_local_adaptation;healthcare_system_critique;pillar_emotional;interdependent_care</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>D1_P12</t>
+          <t>D1_P11</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1187,26 +1179,26 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>2629</v>
+        <v>9126</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q3;Q5</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>awareness_education;interdependent_care;early_detection_prevention;general_response</t>
+          <t>general_response;balance_multidimensional</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>D1_P13</t>
+          <t>D1_P12</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1225,26 +1217,26 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>265</v>
+        <v>2629</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>general_response</t>
+          <t>awareness_education;interdependent_care;early_detection_prevention;general_response</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>D1_P14</t>
+          <t>D1_P13</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1263,10 +1255,10 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>239</v>
+        <v>265</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -1282,17 +1274,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>D1_P15</t>
+          <t>D1_P14</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>HWCH7AR.docx</t>
+          <t>HWCH6AR.docx</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1301,14 +1293,14 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>12656</v>
+        <v>239</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1320,7 +1312,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>D1_P16</t>
+          <t>D1_P15</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1339,10 +1331,10 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>9365</v>
+        <v>12656</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -1358,7 +1350,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>D1_P17</t>
+          <t>D1_P16</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1377,14 +1369,14 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>6223</v>
+        <v>9365</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4;Q5;Q7</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q6;Q7</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1396,7 +1388,7 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>D1_P18</t>
+          <t>D1_P17</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1415,14 +1407,14 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>3595</v>
+        <v>6223</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q3;Q4;Q5;Q6;Q7</t>
+          <t>Q1;Q2;Q3;Q4;Q5;Q7</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1434,7 +1426,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>D1_P19</t>
+          <t>D1_P18</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1453,14 +1445,14 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>3259</v>
+        <v>3595</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q3;Q6;Q7</t>
+          <t>Q1;Q3;Q4;Q5;Q6;Q7</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1472,7 +1464,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>D1_P20</t>
+          <t>D1_P19</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1491,14 +1483,14 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>2554</v>
+        <v>3259</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Q5;Q6;Q7</t>
+          <t>Q1;Q3;Q6;Q7</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -1510,7 +1502,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>D1_P21</t>
+          <t>D1_P20</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1529,14 +1521,14 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>2475</v>
+        <v>2554</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Q3;Q5</t>
+          <t>Q5;Q6;Q7</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1548,17 +1540,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>D1_P22</t>
+          <t>D1_P21</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>HWCH10AR.docx</t>
+          <t>HWCH7AR.docx</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1570,23 +1562,23 @@
         <v>6</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>811</v>
+        <v>2475</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4</t>
+          <t>Q3;Q5</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>pillar_emotional;pillar_physical;cultural_local_adaptation;general_response;pillar_social</t>
+          <t>general_response</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>D1_P23</t>
+          <t>D1_P22</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1605,10 +1597,10 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>1368</v>
+        <v>811</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -1617,14 +1609,14 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>pillar_emotional;cultural_local_adaptation;pillar_social;pillar_intellectual;medical_model_dominance</t>
+          <t>pillar_emotional;pillar_physical;cultural_local_adaptation;general_response;pillar_social</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>D1_P24</t>
+          <t>D1_P23</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1643,26 +1635,26 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>1060</v>
+        <v>1368</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Q2;Q3;Q4</t>
+          <t>Q1;Q2;Q3;Q4</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>pillar_physical;pillar_intellectual;healthcare_system_critique;awareness_education;professional_identity</t>
+          <t>pillar_emotional;cultural_local_adaptation;pillar_social;pillar_intellectual;medical_model_dominance</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>D1_P25</t>
+          <t>D1_P24</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1681,26 +1673,26 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1005</v>
+        <v>1060</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q3;Q4</t>
+          <t>Q2;Q3;Q4</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>balance_multidimensional;pillar_physical;spiritual_moral_anchor;cultural_local_adaptation;healthcare_worker_wellbeing</t>
+          <t>pillar_physical;pillar_intellectual;healthcare_system_critique;awareness_education;professional_identity</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>D1_P26</t>
+          <t>D1_P25</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -1719,26 +1711,26 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>966</v>
+        <v>1005</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Q1;Q2;Q3;Q4</t>
+          <t>Q1;Q3;Q4</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>general_response;pillar_social;child_rights_inclusion;child_vulnerability;family_support_ecology</t>
+          <t>balance_multidimensional;pillar_physical;spiritual_moral_anchor;cultural_local_adaptation;healthcare_worker_wellbeing</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>D1_P27</t>
+          <t>D1_P26</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -1757,93 +1749,131 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>949</v>
+        <v>966</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Q3;Q4</t>
+          <t>Q1;Q2;Q3;Q4</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>interdependent_care;training_deficit;child_vulnerability;school_clinical_link;balance_multidimensional</t>
+          <t>general_response;pillar_social;child_rights_inclusion;child_vulnerability;family_support_ecology</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>D1_U01</t>
+          <t>D1_P27</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>HWCH0AR.docx</t>
+          <t>HWCH10AR.docx</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>participant</t>
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>166</v>
+        <v>949</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Q3;Q5</t>
+          <t>Q3;Q4</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>general_response</t>
+          <t>interdependent_care;training_deficit;child_vulnerability;school_clinical_link;balance_multidimensional</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>D1_U01</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>HWCH0AR.docx</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>166</v>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Q3;Q5</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>general_response</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>D1_U02</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>HWCH6AR.docx</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>unclear</t>
         </is>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E38" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="F38" s="2" t="n">
         <v>978</v>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Q6</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>general_response</t>
         </is>

</xml_diff>